<commit_message>
Day 1: workbook rows marked Live, Rank Math setup done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZFMxKJAHCj2T5ScZR2y1f
</commit_message>
<xml_diff>
--- a/wealthscale-first-100/package/WealthScale_First_100_Index.xlsx
+++ b/wealthscale-first-100/package/WealthScale_First_100_Index.xlsx
@@ -21,9 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="mmm\ d&quot;, &quot;yyyy"/>
     <numFmt numFmtId="165" formatCode="dddd&quot;, &quot;mmm\ d&quot;, &quot;yyyy"/>
+    <numFmt numFmtId="166" formatCode="mmmm d, yyyy"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -111,7 +112,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -147,6 +148,9 @@
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -635,10 +639,12 @@
       </c>
       <c r="S2" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T2" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T2" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="3" ht="35.05" customHeight="1" s="7">
       <c r="A3" s="9" t="n">
@@ -719,10 +725,12 @@
       </c>
       <c r="S3" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T3" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T3" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="4" ht="35.05" customHeight="1" s="7">
       <c r="A4" s="9" t="n">
@@ -803,10 +811,12 @@
       </c>
       <c r="S4" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T4" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T4" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="5" ht="35.05" customHeight="1" s="7">
       <c r="A5" s="9" t="n">
@@ -887,10 +897,12 @@
       </c>
       <c r="S5" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T5" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T5" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="6" ht="35.05" customHeight="1" s="7">
       <c r="A6" s="9" t="n">
@@ -971,10 +983,12 @@
       </c>
       <c r="S6" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T6" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T6" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="7" ht="35.05" customHeight="1" s="7">
       <c r="A7" s="9" t="n">
@@ -1055,10 +1069,12 @@
       </c>
       <c r="S7" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T7" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T7" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="8" ht="35.05" customHeight="1" s="7">
       <c r="A8" s="9" t="n">
@@ -1143,10 +1159,12 @@
       </c>
       <c r="S8" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T8" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T8" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="9" ht="35.05" customHeight="1" s="7">
       <c r="A9" s="9" t="n">
@@ -1231,10 +1249,12 @@
       </c>
       <c r="S9" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T9" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T9" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="10" ht="35.05" customHeight="1" s="7">
       <c r="A10" s="9" t="n">
@@ -1319,10 +1339,12 @@
       </c>
       <c r="S10" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T10" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T10" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="11" ht="35.05" customHeight="1" s="7">
       <c r="A11" s="9" t="n">
@@ -1407,10 +1429,12 @@
       </c>
       <c r="S11" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T11" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T11" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="12" ht="35.05" customHeight="1" s="7">
       <c r="A12" s="9" t="n">
@@ -1495,10 +1519,12 @@
       </c>
       <c r="S12" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T12" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T12" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="13" ht="35.05" customHeight="1" s="7">
       <c r="A13" s="9" t="n">
@@ -1583,10 +1609,12 @@
       </c>
       <c r="S13" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T13" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T13" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="14" ht="35.05" customHeight="1" s="7">
       <c r="A14" s="9" t="n">
@@ -1671,10 +1699,12 @@
       </c>
       <c r="S14" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T14" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T14" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="15" ht="35.05" customHeight="1" s="7">
       <c r="A15" s="9" t="n">
@@ -1759,10 +1789,12 @@
       </c>
       <c r="S15" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T15" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T15" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="16" ht="35.05" customHeight="1" s="7">
       <c r="A16" s="9" t="n">
@@ -1847,10 +1879,12 @@
       </c>
       <c r="S16" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T16" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T16" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="17" ht="35.05" customHeight="1" s="7">
       <c r="A17" s="9" t="n">
@@ -1935,10 +1969,12 @@
       </c>
       <c r="S17" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T17" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T17" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="18" ht="35.05" customHeight="1" s="7">
       <c r="A18" s="9" t="n">
@@ -2023,10 +2059,12 @@
       </c>
       <c r="S18" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T18" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T18" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="19" ht="23.85" customHeight="1" s="7">
       <c r="A19" s="9" t="n">
@@ -2111,10 +2149,12 @@
       </c>
       <c r="S19" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T19" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T19" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="20" ht="23.85" customHeight="1" s="7">
       <c r="A20" s="9" t="n">
@@ -2199,10 +2239,12 @@
       </c>
       <c r="S20" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T20" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T20" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="21" ht="35.05" customHeight="1" s="7">
       <c r="A21" s="9" t="n">
@@ -2283,10 +2325,12 @@
       </c>
       <c r="S21" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T21" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T21" s="13" t="n">
+        <v>46318</v>
+      </c>
     </row>
     <row r="22" ht="35.05" customHeight="1" s="7">
       <c r="A22" s="9" t="n">

</xml_diff>

<commit_message>
Day 2: 20 pages live, workbook rows marked Live
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZFMxKJAHCj2T5ScZR2y1f
</commit_message>
<xml_diff>
--- a/wealthscale-first-100/package/WealthScale_First_100_Index.xlsx
+++ b/wealthscale-first-100/package/WealthScale_First_100_Index.xlsx
@@ -2415,10 +2415,12 @@
       </c>
       <c r="S22" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T22" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T22" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="23" ht="35.05" customHeight="1" s="7">
       <c r="A23" s="9" t="n">
@@ -2503,10 +2505,12 @@
       </c>
       <c r="S23" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T23" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T23" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="24" ht="35.05" customHeight="1" s="7">
       <c r="A24" s="9" t="n">
@@ -2591,10 +2595,12 @@
       </c>
       <c r="S24" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T24" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T24" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="25" ht="23.85" customHeight="1" s="7">
       <c r="A25" s="9" t="n">
@@ -2679,10 +2685,12 @@
       </c>
       <c r="S25" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T25" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T25" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="26" ht="35.05" customHeight="1" s="7">
       <c r="A26" s="9" t="n">
@@ -2767,10 +2775,12 @@
       </c>
       <c r="S26" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T26" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T26" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="27" ht="35.05" customHeight="1" s="7">
       <c r="A27" s="9" t="n">
@@ -2855,10 +2865,12 @@
       </c>
       <c r="S27" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T27" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T27" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="28" ht="35.05" customHeight="1" s="7">
       <c r="A28" s="9" t="n">
@@ -2943,10 +2955,12 @@
       </c>
       <c r="S28" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T28" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T28" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="29" ht="23.85" customHeight="1" s="7">
       <c r="A29" s="9" t="n">
@@ -3031,10 +3045,12 @@
       </c>
       <c r="S29" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T29" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T29" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="30" ht="35.05" customHeight="1" s="7">
       <c r="A30" s="9" t="n">
@@ -3119,10 +3135,12 @@
       </c>
       <c r="S30" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T30" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T30" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="31" ht="35.05" customHeight="1" s="7">
       <c r="A31" s="9" t="n">
@@ -3207,10 +3225,12 @@
       </c>
       <c r="S31" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T31" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T31" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="32" ht="35.05" customHeight="1" s="7">
       <c r="A32" s="9" t="n">
@@ -3295,10 +3315,12 @@
       </c>
       <c r="S32" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T32" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T32" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="33" ht="35.05" customHeight="1" s="7">
       <c r="A33" s="9" t="n">
@@ -3383,10 +3405,12 @@
       </c>
       <c r="S33" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T33" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T33" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="34" ht="35.05" customHeight="1" s="7">
       <c r="A34" s="9" t="n">
@@ -3471,10 +3495,12 @@
       </c>
       <c r="S34" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T34" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T34" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="35" ht="35.05" customHeight="1" s="7">
       <c r="A35" s="9" t="n">
@@ -3559,10 +3585,12 @@
       </c>
       <c r="S35" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T35" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T35" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="36" ht="35.05" customHeight="1" s="7">
       <c r="A36" s="9" t="n">
@@ -3647,10 +3675,12 @@
       </c>
       <c r="S36" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T36" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T36" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="37" ht="35.05" customHeight="1" s="7">
       <c r="A37" s="9" t="n">
@@ -3735,10 +3765,12 @@
       </c>
       <c r="S37" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T37" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T37" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="38" ht="35.05" customHeight="1" s="7">
       <c r="A38" s="9" t="n">
@@ -3823,10 +3855,12 @@
       </c>
       <c r="S38" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T38" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T38" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="39" ht="35.05" customHeight="1" s="7">
       <c r="A39" s="9" t="n">
@@ -3911,10 +3945,12 @@
       </c>
       <c r="S39" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T39" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T39" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="40" ht="35.05" customHeight="1" s="7">
       <c r="A40" s="9" t="n">
@@ -3999,10 +4035,12 @@
       </c>
       <c r="S40" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T40" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T40" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="41" ht="35.05" customHeight="1" s="7">
       <c r="A41" s="9" t="n">
@@ -4087,10 +4125,12 @@
       </c>
       <c r="S41" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T41" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T41" s="13" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="42" ht="35.05" customHeight="1" s="7">
       <c r="A42" s="9" t="n">

</xml_diff>

<commit_message>
Days 3 and 4: 40 pages live, workbook rows marked Live
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZFMxKJAHCj2T5ScZR2y1f
</commit_message>
<xml_diff>
--- a/wealthscale-first-100/package/WealthScale_First_100_Index.xlsx
+++ b/wealthscale-first-100/package/WealthScale_First_100_Index.xlsx
@@ -4215,10 +4215,12 @@
       </c>
       <c r="S42" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T42" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T42" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="43" ht="35.05" customHeight="1" s="7">
       <c r="A43" s="9" t="n">
@@ -4303,10 +4305,12 @@
       </c>
       <c r="S43" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T43" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T43" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="44" ht="35.05" customHeight="1" s="7">
       <c r="A44" s="9" t="n">
@@ -4391,10 +4395,12 @@
       </c>
       <c r="S44" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T44" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T44" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="45" ht="35.05" customHeight="1" s="7">
       <c r="A45" s="9" t="n">
@@ -4479,10 +4485,12 @@
       </c>
       <c r="S45" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T45" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T45" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="46" ht="35.05" customHeight="1" s="7">
       <c r="A46" s="9" t="n">
@@ -4567,10 +4575,12 @@
       </c>
       <c r="S46" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T46" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T46" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="47" ht="35.05" customHeight="1" s="7">
       <c r="A47" s="9" t="n">
@@ -4655,10 +4665,12 @@
       </c>
       <c r="S47" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T47" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T47" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="48" ht="23.85" customHeight="1" s="7">
       <c r="A48" s="9" t="n">
@@ -4743,10 +4755,12 @@
       </c>
       <c r="S48" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T48" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T48" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="49" ht="35.05" customHeight="1" s="7">
       <c r="A49" s="9" t="n">
@@ -4831,10 +4845,12 @@
       </c>
       <c r="S49" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T49" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T49" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="50" ht="35.05" customHeight="1" s="7">
       <c r="A50" s="9" t="n">
@@ -4919,10 +4935,12 @@
       </c>
       <c r="S50" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T50" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T50" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="51" ht="35.05" customHeight="1" s="7">
       <c r="A51" s="9" t="n">
@@ -5007,10 +5025,12 @@
       </c>
       <c r="S51" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T51" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T51" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="52" ht="35.05" customHeight="1" s="7">
       <c r="A52" s="9" t="n">
@@ -5095,10 +5115,12 @@
       </c>
       <c r="S52" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T52" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T52" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="53" ht="35.05" customHeight="1" s="7">
       <c r="A53" s="9" t="n">
@@ -5183,10 +5205,12 @@
       </c>
       <c r="S53" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T53" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T53" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="54" ht="35.05" customHeight="1" s="7">
       <c r="A54" s="9" t="n">
@@ -5271,10 +5295,12 @@
       </c>
       <c r="S54" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T54" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T54" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="55" ht="35.05" customHeight="1" s="7">
       <c r="A55" s="9" t="n">
@@ -5359,10 +5385,12 @@
       </c>
       <c r="S55" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T55" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T55" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="56" ht="35.05" customHeight="1" s="7">
       <c r="A56" s="9" t="n">
@@ -5447,10 +5475,12 @@
       </c>
       <c r="S56" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T56" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T56" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="57" ht="35.05" customHeight="1" s="7">
       <c r="A57" s="9" t="n">
@@ -5535,10 +5565,12 @@
       </c>
       <c r="S57" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T57" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T57" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="58" ht="35.05" customHeight="1" s="7">
       <c r="A58" s="9" t="n">
@@ -5623,10 +5655,12 @@
       </c>
       <c r="S58" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T58" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T58" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="59" ht="35.05" customHeight="1" s="7">
       <c r="A59" s="9" t="n">
@@ -5711,10 +5745,12 @@
       </c>
       <c r="S59" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T59" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T59" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="60" ht="35.05" customHeight="1" s="7">
       <c r="A60" s="9" t="n">
@@ -5799,10 +5835,12 @@
       </c>
       <c r="S60" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T60" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T60" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="61" ht="35.05" customHeight="1" s="7">
       <c r="A61" s="9" t="n">
@@ -5887,10 +5925,12 @@
       </c>
       <c r="S61" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T61" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T61" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="62" ht="35.05" customHeight="1" s="7">
       <c r="A62" s="9" t="n">
@@ -5975,10 +6015,12 @@
       </c>
       <c r="S62" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T62" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T62" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="63" ht="35.05" customHeight="1" s="7">
       <c r="A63" s="9" t="n">
@@ -6063,10 +6105,12 @@
       </c>
       <c r="S63" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T63" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T63" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="64" ht="35.05" customHeight="1" s="7">
       <c r="A64" s="9" t="n">
@@ -6151,10 +6195,12 @@
       </c>
       <c r="S64" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T64" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T64" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="65" ht="35.05" customHeight="1" s="7">
       <c r="A65" s="9" t="n">
@@ -6239,10 +6285,12 @@
       </c>
       <c r="S65" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T65" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T65" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="66" ht="35.05" customHeight="1" s="7">
       <c r="A66" s="9" t="n">
@@ -6327,10 +6375,12 @@
       </c>
       <c r="S66" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T66" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T66" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="67" ht="35.05" customHeight="1" s="7">
       <c r="A67" s="9" t="n">
@@ -6415,10 +6465,12 @@
       </c>
       <c r="S67" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T67" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T67" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="68" ht="35.05" customHeight="1" s="7">
       <c r="A68" s="9" t="n">
@@ -6503,10 +6555,12 @@
       </c>
       <c r="S68" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T68" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T68" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="69" ht="35.05" customHeight="1" s="7">
       <c r="A69" s="9" t="n">
@@ -6591,10 +6645,12 @@
       </c>
       <c r="S69" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T69" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T69" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="70" ht="35.05" customHeight="1" s="7">
       <c r="A70" s="9" t="n">
@@ -6679,10 +6735,12 @@
       </c>
       <c r="S70" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T70" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T70" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="71" ht="35.05" customHeight="1" s="7">
       <c r="A71" s="9" t="n">
@@ -6767,10 +6825,12 @@
       </c>
       <c r="S71" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T71" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T71" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="72" ht="35.05" customHeight="1" s="7">
       <c r="A72" s="9" t="n">
@@ -6855,10 +6915,12 @@
       </c>
       <c r="S72" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T72" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T72" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="73" ht="35.05" customHeight="1" s="7">
       <c r="A73" s="9" t="n">
@@ -6943,10 +7005,12 @@
       </c>
       <c r="S73" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T73" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T73" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="74" ht="35.05" customHeight="1" s="7">
       <c r="A74" s="9" t="n">
@@ -7031,10 +7095,12 @@
       </c>
       <c r="S74" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T74" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T74" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="75" ht="35.05" customHeight="1" s="7">
       <c r="A75" s="9" t="n">
@@ -7119,10 +7185,12 @@
       </c>
       <c r="S75" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T75" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T75" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="76" ht="35.05" customHeight="1" s="7">
       <c r="A76" s="9" t="n">
@@ -7207,10 +7275,12 @@
       </c>
       <c r="S76" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T76" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T76" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="77" ht="35.05" customHeight="1" s="7">
       <c r="A77" s="9" t="n">
@@ -7295,10 +7365,12 @@
       </c>
       <c r="S77" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T77" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T77" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="78" ht="35.05" customHeight="1" s="7">
       <c r="A78" s="9" t="n">
@@ -7383,10 +7455,12 @@
       </c>
       <c r="S78" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T78" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T78" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="79" ht="35.05" customHeight="1" s="7">
       <c r="A79" s="9" t="n">
@@ -7471,10 +7545,12 @@
       </c>
       <c r="S79" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T79" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T79" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="80" ht="35.05" customHeight="1" s="7">
       <c r="A80" s="9" t="n">
@@ -7559,10 +7635,12 @@
       </c>
       <c r="S80" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T80" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T80" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="81" ht="35.05" customHeight="1" s="7">
       <c r="A81" s="9" t="n">
@@ -7647,10 +7725,12 @@
       </c>
       <c r="S81" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="T81" s="10" t="n"/>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="T81" s="13" t="n">
+        <v>46321</v>
+      </c>
     </row>
     <row r="82" ht="35.05" customHeight="1" s="7">
       <c r="A82" s="9" t="n">

</xml_diff>